<commit_message>
feat: editable rollover from Sept, real-time solvency engine, clean debt slate, and gmail automation update
</commit_message>
<xml_diff>
--- a/Dhruv_Financial_OS_Setup_Template.xlsx
+++ b/Dhruv_Financial_OS_Setup_Template.xlsx
@@ -107,13 +107,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -495,14 +495,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="41" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -542,73 +542,98 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>HDFC Bank Account</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Bank</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
+          <t>Opening Rollover (B/F from September)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Rollover</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
         <v>25000</v>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Primary Salary Account, Debits, Rent &amp; Bills</t>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Surplus cash carried forward from previous month</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
+          <t>HDFC Bank Account</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Bank</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Primary Salary Account, Debits, Rent &amp; Bills</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
           <t>Kotak Bank Account</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Bank</t>
         </is>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="C5" s="5" t="n">
         <v>10000</v>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Stock Trading &amp; Investment Liquidity Account</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>Cash in Hand</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C6" s="7" t="n">
         <v>1000</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D6" s="8" t="inlineStr">
         <is>
           <t>2026-10-01</t>
         </is>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Physical Wallet &amp; Cash Expenses</t>
         </is>
@@ -715,46 +740,46 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>American Express Credit Card</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Amex</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Amex</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>4001</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>360000</v>
       </c>
       <c r="F3" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="H3" s="4" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>10/28</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr"/>
+      <c r="K3" s="4" t="inlineStr"/>
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>MRCC Points, Fuel waiver, Milestones</t>
         </is>
@@ -807,46 +832,46 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>ICICI - Coral Credit Card</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>ICICI</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Visa</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>2004</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>100000</v>
       </c>
       <c r="F5" s="9" t="n">
         <v>21</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="3" t="inlineStr">
         <is>
           <t>2026-10-10</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="H5" s="4" t="inlineStr"/>
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>08/28</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="J5" s="4" t="inlineStr"/>
+      <c r="K5" s="4" t="inlineStr"/>
+      <c r="L5" s="4" t="inlineStr">
         <is>
           <t>Airport Lounge, BMS Buy 1 Get 1</t>
         </is>
@@ -899,46 +924,46 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>HDFC - Money Back Plus Credit Card</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>HDFC</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>Visa</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>1005</t>
         </is>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>69000</v>
       </c>
       <c r="F7" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>11/27</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="J7" s="4" t="inlineStr"/>
+      <c r="K7" s="4" t="inlineStr"/>
+      <c r="L7" s="4" t="inlineStr">
         <is>
           <t>HDFC Core Rewards, SmartBuy cashback</t>
         </is>
@@ -1049,25 +1074,25 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Dad</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Family Ledger</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>They Owe Me</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" s="4" t="inlineStr">
         <is>
           <t>Family shared expenses and monthly settles</t>
         </is>
@@ -1112,17 +1137,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
     <col width="25" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1171,74 +1196,6 @@
       <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>iPhone 17 Pro EMI</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>ICICI - Coral Credit Card</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>135000</v>
-      </c>
-      <c r="D3" s="9" t="n">
-        <v>11250</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="G3" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Watch EMI</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>ICICI - Coral Credit Card</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="n">
-        <v>8418.07</v>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>2894.6</v>
-      </c>
-      <c r="E4" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="G4" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Active (Final payoff in Oct)</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1219,7 @@
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1295,20 +1252,20 @@
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Food &amp; Dining</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="C3" s="4" t="n">
+      <c r="C3" s="5" t="n">
         <v>8000</v>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>🍔 Swiggy, Zomato, Restaurants, Cafes</t>
         </is>
@@ -1335,20 +1292,20 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Fuel &amp; Conveyance</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>4000</v>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>⛽ Petrol, Uber, Auto, Fastag</t>
         </is>
@@ -1375,20 +1332,20 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Bills &amp; Utilities</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Expense</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>💡 Electricity, Wi-Fi, Mobile recharge</t>
         </is>
@@ -1417,20 +1374,20 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro EMI</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
+          <t>Loan / EMI Payment</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Debt</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>11250</v>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>📱 Coral Card Monthly EMI</t>
+          <t>💳 General EMI / Loan (Add specific when they occur)</t>
         </is>
       </c>
     </row>
@@ -1455,20 +1412,20 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Kotak Transfer</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Income</t>
         </is>
       </c>
-      <c r="C11" s="4" t="n">
+      <c r="C11" s="5" t="n">
         <v>9439</v>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>📈 Liquidity / Trading pull-in</t>
         </is>

</xml_diff>

<commit_message>
feat: configure all 7 credit cards with exact statement and due schedules, add CheQ AU card, and update Excel template
</commit_message>
<xml_diff>
--- a/Dhruv_Financial_OS_Setup_Template.xlsx
+++ b/Dhruv_Financial_OS_Setup_Template.xlsx
@@ -653,11 +653,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="51" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
@@ -667,7 +667,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="47" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -747,7 +747,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Amex</t>
+          <t>American Express</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -781,19 +781,19 @@
       <c r="K3" s="4" t="inlineStr"/>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>MRCC Points, Fuel waiver, Milestones</t>
+          <t>8th cycle, Due 26th of month</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>ICICI - Amazon Pay Credit Card</t>
+          <t>ICICI Bank Credit Card (Coral)</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>ICICI</t>
+          <t>ICICI Bank</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -803,43 +803,43 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>3002</t>
+          <t>2004</t>
         </is>
       </c>
       <c r="E4" s="7" t="n">
-        <v>120000</v>
+        <v>100000</v>
       </c>
       <c r="F4" s="10" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr"/>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>12/27</t>
+          <t>08/28</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr"/>
       <c r="K4" s="6" t="inlineStr"/>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>5% Unlimited Amazon Cashback</t>
+          <t>2nd-3rd cycle, Due 19th-20th of month</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>ICICI - Coral Credit Card</t>
+          <t>Amazon Pay ICICI Bank Credit Card</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ICICI</t>
+          <t>ICICI Bank</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -849,89 +849,89 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2004</t>
+          <t>3002</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>100000</v>
+        <v>120000</v>
       </c>
       <c r="F5" s="9" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr"/>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>08/28</t>
+          <t>12/27</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr"/>
       <c r="K5" s="4" t="inlineStr"/>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Airport Lounge, BMS Buy 1 Get 1</t>
+          <t>2nd-3rd cycle, Due 19th of month</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>Roar CC RuPay</t>
+          <t>HDFC Bank Pixel Play Credit Card</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Roar</t>
+          <t>HDFC Bank</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>RuPay</t>
+          <t>Visa</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>5003</t>
+          <t>9006</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
-        <v>150000</v>
+        <v>15000</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="H6" s="6" t="inlineStr"/>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>05/29</t>
+          <t>04/28</t>
         </is>
       </c>
       <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="6" t="inlineStr"/>
       <c r="L6" s="6" t="inlineStr">
         <is>
-          <t>UPI on Credit Card, Reward Points</t>
+          <t>1st-2nd cycle, Due 21st of month</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>HDFC - Money Back Plus Credit Card</t>
+          <t>HDFC Bank MoneyBack+ Credit Card</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>HDFC</t>
+          <t>HDFC Bank</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -948,11 +948,11 @@
         <v>69000</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-11-02</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr"/>
@@ -965,53 +965,99 @@
       <c r="K7" s="4" t="inlineStr"/>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>HDFC Core Rewards, SmartBuy cashback</t>
+          <t>12th cycle, Due 1st-2nd of following month</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>HDFC - Pixel Play Credit Card</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>HDFC</t>
+          <t>Roarbank Credit Card (Unity Small Finance Bank)</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Unity / Roar</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Visa</t>
+          <t>RuPay</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>9006</t>
+          <t>5003</t>
         </is>
       </c>
       <c r="E8" s="7" t="n">
-        <v>15000</v>
+        <v>150000</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="H8" s="6" t="inlineStr"/>
       <c r="I8" s="8" t="inlineStr">
         <is>
-          <t>04/28</t>
+          <t>05/29</t>
         </is>
       </c>
       <c r="J8" s="6" t="inlineStr"/>
       <c r="K8" s="6" t="inlineStr"/>
       <c r="L8" s="8" t="inlineStr">
         <is>
-          <t>Digital Custom Cashbacks (Zomato/Blinkit)</t>
+          <t>30th/1st cycle, Due 28th of following month</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>CheQ Credit Card (AU Small Finance Bank)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>AU Small Finance Bank</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Visa</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>7007</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F9" s="9" t="n">
+        <v>24</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-13</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>09/29</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr"/>
+      <c r="K9" s="4" t="inlineStr"/>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>24th cycle, Due 13th of following month</t>
         </is>
       </c>
     </row>

</xml_diff>